<commit_message>
Promociones: cantidad minima, precio con decimales y grupos divididos
</commit_message>
<xml_diff>
--- a/excel/PROMOCIONES.xlsx
+++ b/excel/PROMOCIONES.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>CODIGO_PRODUCTO</t>
   </si>
@@ -41,13 +41,19 @@
     <t>GRUPOS</t>
   </si>
   <si>
-    <t>GRUPO_SINPAR</t>
-  </si>
-  <si>
     <t>F</t>
   </si>
   <si>
-    <t>SPDARC115160222</t>
+    <t>CANTIDAD_MINIMA</t>
+  </si>
+  <si>
+    <t>DOSF1601</t>
+  </si>
+  <si>
+    <t>PREMIUM TOP</t>
+  </si>
+  <si>
+    <t>PREMIUM</t>
   </si>
 </sst>
 </file>
@@ -83,9 +89,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -366,13 +373,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" customWidth="1"/>
+    <col min="6" max="6" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -388,22 +397,48 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2">
-        <v>432.24099999999999</v>
+        <v>5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2719.5</v>
       </c>
       <c r="D2" s="1">
-        <v>45657</v>
+        <v>46289</v>
       </c>
       <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2719.5</v>
+      </c>
+      <c r="D3" s="1">
+        <v>46289</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Promociones: cinta en las tarjetas segun grupo y cantidad minima
</commit_message>
<xml_diff>
--- a/excel/PROMOCIONES.xlsx
+++ b/excel/PROMOCIONES.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>CODIGO_PRODUCTO</t>
   </si>
@@ -50,10 +50,7 @@
     <t>DOSF1601</t>
   </si>
   <si>
-    <t>PREMIUM TOP</t>
-  </si>
-  <si>
-    <t>PREMIUM</t>
+    <t>PREMIUM.PREMIUM TOP</t>
   </si>
 </sst>
 </file>
@@ -373,11 +370,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="5" max="5" width="21.140625" customWidth="1"/>
+    <col min="5" max="5" width="25.85546875" customWidth="1"/>
     <col min="6" max="6" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -421,26 +418,6 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2719.5</v>
-      </c>
-      <c r="D3" s="1">
-        <v>46289</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3">
-        <v>75</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>